<commit_message>
starting 26/27 fpl in a week!
</commit_message>
<xml_diff>
--- a/docs/fpl_scoring_2025_26.xlsx
+++ b/docs/fpl_scoring_2025_26.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\fpl_analytics\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F18A561-A501-4332-8678-2F53EBDF46E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41C1DACB-00EF-4B8C-89D4-068DC4F4AF5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="48">
   <si>
     <t>Fantasy Premier League — 2025/26 Scoring Rules</t>
   </si>
@@ -158,6 +158,12 @@
   </si>
   <si>
     <t>xa, chances_created, xgi, accurate_crosses, accurate_long_balls, final_third_passes, touches_opposition_box, corners, touches…xa + chances_created + accurate_crosses + position</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CASE WHEN team_goals_conceded = 0 AND minutes_played &gt;= 60 THEN 1 ELSE 0 END </t>
+  </si>
+  <si>
+    <t>cbit, cbitr, saves, xgot_faced, blocks + clearances + interceptions, tackles, teams_goals_conceeded, opponent elo (figure out), strength_defence_home, strength_defence_away</t>
   </si>
 </sst>
 </file>
@@ -649,7 +655,7 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
-    <col min="2" max="2" width="58" customWidth="1"/>
+    <col min="2" max="2" width="65.109375" customWidth="1"/>
     <col min="3" max="3" width="10" customWidth="1"/>
     <col min="4" max="4" width="22" customWidth="1"/>
     <col min="5" max="5" width="46.88671875" customWidth="1"/>
@@ -830,7 +836,7 @@
       <c r="C13" s="11"/>
       <c r="D13" s="11"/>
     </row>
-    <row r="14" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
         <v>17</v>
       </c>
@@ -842,6 +848,12 @@
       </c>
       <c r="D14" s="7" t="s">
         <v>12</v>
+      </c>
+      <c r="E14" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="F14" s="17" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>